<commit_message>
feat: add feeder cable rules W12814-W12829, 3-line structured prompt format, and feeder mapping migration
</commit_message>
<xml_diff>
--- a/backend/uploads/price_list_1.xlsx
+++ b/backend/uploads/price_list_1.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule of Rates" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule of Rates'!$A$3:$H$179</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Schedule of Rates'!$A$3:$H$177</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H180"/>
+  <dimension ref="A1:H178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2963,17 +2963,13 @@
         <v>189.6</v>
       </c>
       <c r="F83" s="17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G83" s="18">
         <f>E83*F83</f>
         <v/>
       </c>
-      <c r="H83" s="13" t="inlineStr">
-        <is>
-          <t>3x ERICSSON BB6630, 1x ERICSSON DUW 30 01, 2x ERICSSON R503, 1x FIBRE MANAGEMENT TRAY</t>
-        </is>
-      </c>
+      <c r="H83" s="13" t="inlineStr"/>
     </row>
     <row r="84" ht="26" customHeight="1">
       <c r="A84" s="7" t="inlineStr">
@@ -3151,11 +3147,7 @@
         <f>E89*F89</f>
         <v/>
       </c>
-      <c r="H89" s="13" t="inlineStr">
-        <is>
-          <t>1x ERICSSON RP6672</t>
-        </is>
-      </c>
+      <c r="H89" s="13" t="inlineStr"/>
     </row>
     <row r="90" ht="40" customHeight="1">
       <c r="A90" s="7" t="inlineStr">
@@ -3240,17 +3232,13 @@
         <v>188.5</v>
       </c>
       <c r="F92" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G92" s="18">
         <f>E92*F92</f>
         <v/>
       </c>
-      <c r="H92" s="13" t="inlineStr">
-        <is>
-          <t>1x ERICSSON R6675 ROUTER to be relocated from RT/1/1/6 to RT/1/1/29, 1x SLIDEOUT FIBRE MANAGEMENT TRAY to be relocated from RT/1/1/29 to RT/1/1/30</t>
-        </is>
-      </c>
+      <c r="H92" s="13" t="inlineStr"/>
     </row>
     <row r="93" ht="26" customHeight="1">
       <c r="A93" s="7" t="inlineStr">
@@ -3572,33 +3560,37 @@
       <c r="H103" s="7" t="inlineStr"/>
     </row>
     <row r="104" ht="26" customHeight="1">
-      <c r="A104" s="7" t="inlineStr">
+      <c r="A104" s="13" t="inlineStr">
         <is>
           <t>R13169</t>
         </is>
       </c>
-      <c r="B104" s="8" t="inlineStr">
+      <c r="B104" s="14" t="inlineStr">
         <is>
           <t>Removal and Recover internal Filter or Combiner</t>
         </is>
       </c>
-      <c r="C104" s="9" t="inlineStr"/>
-      <c r="D104" s="9" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="E104" s="10" t="n">
+      <c r="C104" s="15" t="inlineStr">
+        <is>
+          <t>REMOVE</t>
+        </is>
+      </c>
+      <c r="D104" s="15" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="n">
         <v>72.09999999999999</v>
       </c>
-      <c r="F104" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G104" s="12">
+      <c r="F104" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G104" s="18">
         <f>E104*F104</f>
         <v/>
       </c>
-      <c r="H104" s="7" t="inlineStr"/>
+      <c r="H104" s="13" t="inlineStr"/>
     </row>
     <row r="105" ht="26" customHeight="1">
       <c r="A105" s="7" t="inlineStr">
@@ -4094,70 +4086,62 @@
       <c r="H121" s="7" t="inlineStr"/>
     </row>
     <row r="122" ht="26" customHeight="1">
-      <c r="A122" s="13" t="inlineStr">
+      <c r="A122" s="7" t="inlineStr">
         <is>
           <t>ST002</t>
         </is>
       </c>
-      <c r="B122" s="14" t="inlineStr">
+      <c r="B122" s="8" t="inlineStr">
         <is>
           <t>RRU installed in shelter</t>
         </is>
       </c>
-      <c r="C122" s="15" t="inlineStr">
-        <is>
-          <t>INSTALL</t>
-        </is>
-      </c>
-      <c r="D122" s="15" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="E122" s="16" t="n">
+      <c r="C122" s="9" t="inlineStr"/>
+      <c r="D122" s="9" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="E122" s="10" t="n">
         <v>475</v>
       </c>
-      <c r="F122" s="17" t="n">
-        <v>6</v>
-      </c>
-      <c r="G122" s="18">
+      <c r="F122" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" s="12">
         <f>E122*F122</f>
         <v/>
       </c>
-      <c r="H122" s="13" t="inlineStr"/>
+      <c r="H122" s="7" t="inlineStr"/>
     </row>
     <row r="123" ht="26" customHeight="1">
-      <c r="A123" s="13" t="inlineStr">
+      <c r="A123" s="7" t="inlineStr">
         <is>
           <t>ST003</t>
         </is>
       </c>
-      <c r="B123" s="14" t="inlineStr">
+      <c r="B123" s="8" t="inlineStr">
         <is>
           <t>RRU recovery from shelter</t>
         </is>
       </c>
-      <c r="C123" s="15" t="inlineStr">
-        <is>
-          <t>REMOVE</t>
-        </is>
-      </c>
-      <c r="D123" s="15" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="E123" s="16" t="n">
+      <c r="C123" s="9" t="inlineStr"/>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="E123" s="10" t="n">
         <v>225</v>
       </c>
-      <c r="F123" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="G123" s="18">
+      <c r="F123" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" s="12">
         <f>E123*F123</f>
         <v/>
       </c>
-      <c r="H123" s="13" t="inlineStr"/>
+      <c r="H123" s="7" t="inlineStr"/>
     </row>
     <row r="124" ht="26" customHeight="1">
       <c r="A124" s="7" t="inlineStr">
@@ -4624,62 +4608,70 @@
       <c r="H139" s="7" t="inlineStr"/>
     </row>
     <row r="140" ht="26" customHeight="1">
-      <c r="A140" s="7" t="inlineStr">
+      <c r="A140" s="13" t="inlineStr">
         <is>
           <t>ST007</t>
         </is>
       </c>
-      <c r="B140" s="8" t="inlineStr">
+      <c r="B140" s="14" t="inlineStr">
         <is>
           <t>FIM and waste management</t>
         </is>
       </c>
-      <c r="C140" s="9" t="inlineStr"/>
-      <c r="D140" s="9" t="inlineStr">
+      <c r="C140" s="15" t="inlineStr">
+        <is>
+          <t>MANAGE</t>
+        </is>
+      </c>
+      <c r="D140" s="15" t="inlineStr">
         <is>
           <t>per site</t>
         </is>
       </c>
-      <c r="E140" s="10" t="n">
+      <c r="E140" s="16" t="n">
         <v>860</v>
       </c>
-      <c r="F140" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G140" s="12">
+      <c r="F140" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G140" s="18">
         <f>E140*F140</f>
         <v/>
       </c>
-      <c r="H140" s="7" t="inlineStr"/>
+      <c r="H140" s="13" t="inlineStr"/>
     </row>
     <row r="141" ht="26" customHeight="1">
-      <c r="A141" s="7" t="inlineStr">
+      <c r="A141" s="13" t="inlineStr">
         <is>
           <t>W13398</t>
         </is>
       </c>
-      <c r="B141" s="8" t="inlineStr">
+      <c r="B141" s="14" t="inlineStr">
         <is>
           <t>Tier 2 Tower Inspections BAU when completing Build</t>
         </is>
       </c>
-      <c r="C141" s="9" t="inlineStr"/>
-      <c r="D141" s="9" t="inlineStr">
+      <c r="C141" s="15" t="inlineStr">
+        <is>
+          <t>INSPECT</t>
+        </is>
+      </c>
+      <c r="D141" s="15" t="inlineStr">
         <is>
           <t>per site</t>
         </is>
       </c>
-      <c r="E141" s="10" t="n">
+      <c r="E141" s="16" t="n">
         <v>329</v>
       </c>
-      <c r="F141" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G141" s="12">
+      <c r="F141" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G141" s="18">
         <f>E141*F141</f>
         <v/>
       </c>
-      <c r="H141" s="7" t="inlineStr"/>
+      <c r="H141" s="13" t="inlineStr"/>
     </row>
     <row r="142" ht="26" customHeight="1">
       <c r="A142" s="7" t="inlineStr">
@@ -5561,17 +5553,13 @@
         <v>97.5</v>
       </c>
       <c r="F172" s="17" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G172" s="18">
         <f>E172*F172</f>
         <v/>
       </c>
-      <c r="H172" s="13" t="inlineStr">
-        <is>
-          <t>Reuse 12x RFS LCF78-50JA/J and 3x W&amp;B HYBRID CABLE 7/8". As per drawing notes, PIM test is required on existing feeders.</t>
-        </is>
-      </c>
+      <c r="H172" s="13" t="inlineStr"/>
     </row>
     <row r="173" ht="54" customHeight="1">
       <c r="A173" s="13" t="inlineStr">
@@ -5604,48 +5592,36 @@
         <f>E173*F173</f>
         <v/>
       </c>
-      <c r="H173" s="13" t="inlineStr">
-        <is>
-          <t>3 technology sectors (3x 4G sectors, 3x 5G sectors) first carrier testing</t>
-        </is>
-      </c>
+      <c r="H173" s="13" t="inlineStr"/>
     </row>
     <row r="174" ht="54" customHeight="1">
-      <c r="A174" s="13" t="inlineStr">
+      <c r="A174" s="7" t="inlineStr">
         <is>
           <t>W13400</t>
         </is>
       </c>
-      <c r="B174" s="14" t="inlineStr">
+      <c r="B174" s="8" t="inlineStr">
         <is>
           <t>Testing of 4G/5G Installation using Blackbird App including all required Call / Data Tests (extra over first carrier per sector for each subsequent carrier per sector)</t>
         </is>
       </c>
-      <c r="C174" s="15" t="inlineStr">
-        <is>
-          <t>TEST</t>
-        </is>
-      </c>
-      <c r="D174" s="15" t="inlineStr">
+      <c r="C174" s="9" t="inlineStr"/>
+      <c r="D174" s="9" t="inlineStr">
         <is>
           <t>per sector / carrier</t>
         </is>
       </c>
-      <c r="E174" s="16" t="n">
+      <c r="E174" s="10" t="n">
         <v>91</v>
       </c>
-      <c r="F174" s="17" t="n">
-        <v>18</v>
-      </c>
-      <c r="G174" s="18">
+      <c r="F174" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G174" s="12">
         <f>E174*F174</f>
         <v/>
       </c>
-      <c r="H174" s="13" t="inlineStr">
-        <is>
-          <t>18 extra-over carriers across 6 antennas</t>
-        </is>
-      </c>
+      <c r="H174" s="7" t="inlineStr"/>
     </row>
     <row r="175" ht="24" customHeight="1">
       <c r="A175" s="5" t="inlineStr">
@@ -5669,7 +5645,7 @@
       </c>
       <c r="B176" s="14" t="inlineStr">
         <is>
-          <t>PROPOSED POLE Ø139.7x5.0Thk CHS, 3216mm LONG</t>
+          <t>EME CHAIN BARRIER SUPPORT WITH HILTI ANCHORS</t>
         </is>
       </c>
       <c r="C176" s="15" t="inlineStr">
@@ -5686,7 +5662,7 @@
         <v>0</v>
       </c>
       <c r="F176" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G176" s="18">
         <f>E176*F176</f>
@@ -5694,7 +5670,7 @@
       </c>
       <c r="H176" s="13" t="inlineStr">
         <is>
-          <t>Estimator need to fill: Proposed structural steel pole P1, Ø139.7x5.0Thk CHS, 3216mm long as per Member Schedule (Sheet 23).</t>
+          <t>Estimator need to fill: Proposed EME chain barrier support with 4 Nos Hilti anchors (3 off), Drawing sheet T8-7</t>
         </is>
       </c>
     </row>
@@ -5706,12 +5682,12 @@
       </c>
       <c r="B177" s="14" t="inlineStr">
         <is>
-          <t>PROPOSED POLE Ø139.7x5.0Thk CHS, 2494mm LONG</t>
+          <t>PLINTH DEMOLITION AND RECONSTRUCTION</t>
         </is>
       </c>
       <c r="C177" s="15" t="inlineStr">
         <is>
-          <t>INSTALL</t>
+          <t>MODIFIED</t>
         </is>
       </c>
       <c r="D177" s="15" t="inlineStr">
@@ -5723,7 +5699,7 @@
         <v>0</v>
       </c>
       <c r="F177" s="17" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G177" s="18">
         <f>E177*F177</f>
@@ -5731,103 +5707,29 @@
       </c>
       <c r="H177" s="13" t="inlineStr">
         <is>
-          <t>Estimator need to fill: Proposed structural steel pole P2, Ø139.7x5.0Thk CHS, 2494mm long as per Member Schedule (Sheet 23).</t>
+          <t>Estimator need to fill: Existing diagonal brace connection plinths (4-off) demolition and replacement with new plinths, waterproofing, and Hilti chemical anchors, Drawing sheet T3-8</t>
         </is>
       </c>
     </row>
     <row r="178" ht="26" customHeight="1">
-      <c r="A178" s="13" t="inlineStr">
-        <is>
-          <t>UNQUOTED</t>
-        </is>
-      </c>
-      <c r="B178" s="14" t="inlineStr">
-        <is>
-          <t>PROPOSED ANTENNA MOUNT Ø76.1x4.5Thk CHS, 2800mm LONG</t>
-        </is>
-      </c>
-      <c r="C178" s="15" t="inlineStr">
-        <is>
-          <t>INSTALL</t>
-        </is>
-      </c>
-      <c r="D178" s="15" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="E178" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F178" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="G178" s="18">
-        <f>E178*F178</f>
-        <v/>
-      </c>
-      <c r="H178" s="13" t="inlineStr">
-        <is>
-          <t>Estimator need to fill: Proposed antenna mount AM1, Ø76.1x4.5Thk CHS, 2800mm long as per Member Schedule (Sheet 23).</t>
-        </is>
-      </c>
-    </row>
-    <row r="179" ht="26" customHeight="1">
-      <c r="A179" s="13" t="inlineStr">
-        <is>
-          <t>UNQUOTED</t>
-        </is>
-      </c>
-      <c r="B179" s="14" t="inlineStr">
-        <is>
-          <t>PROPOSED EME CHAIN BARRIER SUPPORT WITH 4 Nos HILTI ANCHORS</t>
-        </is>
-      </c>
-      <c r="C179" s="15" t="inlineStr">
-        <is>
-          <t>INSTALL</t>
-        </is>
-      </c>
-      <c r="D179" s="15" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="E179" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F179" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="G179" s="18">
-        <f>E179*F179</f>
-        <v/>
-      </c>
-      <c r="H179" s="13" t="inlineStr">
-        <is>
-          <t>Estimator need to fill: Proposed EME chain barrier support with 4 Nos Hilti anchors as per Member Schedule (Sheet 24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="180" ht="26" customHeight="1">
-      <c r="A180" s="19" t="n"/>
-      <c r="B180" s="20" t="inlineStr">
+      <c r="A178" s="19" t="n"/>
+      <c r="B178" s="20" t="inlineStr">
         <is>
           <t>TOTAL ESTIMATED COST (EXCLUDING GST)</t>
         </is>
       </c>
-      <c r="C180" s="19" t="n"/>
-      <c r="D180" s="19" t="n"/>
-      <c r="E180" s="19" t="n"/>
-      <c r="F180" s="19" t="n"/>
-      <c r="G180" s="21">
-        <f>SUM(G4:G179)</f>
-        <v/>
-      </c>
-      <c r="H180" s="19" t="n"/>
+      <c r="C178" s="19" t="n"/>
+      <c r="D178" s="19" t="n"/>
+      <c r="E178" s="19" t="n"/>
+      <c r="F178" s="19" t="n"/>
+      <c r="G178" s="21">
+        <f>SUM(G4:G177)</f>
+        <v/>
+      </c>
+      <c r="H178" s="19" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H179"/>
+  <autoFilter ref="A3:H177"/>
   <mergeCells count="4">
     <mergeCell ref="A175:H175"/>
     <mergeCell ref="A4:H4"/>

</xml_diff>